<commit_message>
Add 990542 photo; feature trolley jack 205336; hide 205264
Wire new product photo public/products/990542.jpg. Apply spreadsheet edits:
set 205336 (215N air/hydraulic trolley jack) Name Override + Description and
Featured=Y; hide 205264 (Add to site=N), dropping its image mapping.

Also restores 109 Air Tools short descriptions that an Excel save had blanked
in products.xlsx (re-applied via the blank-only draft step; tyre-tube and
manual edits untouched).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/products.xlsx
+++ b/data/products.xlsx
@@ -16043,7 +16043,7 @@
         <v/>
       </c>
       <c r="O294" t="str">
-        <v>Y</v>
+        <v>N</v>
       </c>
       <c r="P294" t="str">
         <v>N</v>
@@ -16052,7 +16052,7 @@
         <v/>
       </c>
     </row>
-    <row r="295">
+    <row r="295" xml:space="preserve">
       <c r="A295" t="str">
         <v>p321</v>
       </c>
@@ -16063,13 +16063,21 @@
         <v>Jack Air/Hyd 40/20T YAK215N</v>
       </c>
       <c r="D295" t="str">
-        <v/>
+        <v>215N, Air/Hydraulic 2-Stage Trolley Jack (40/20T)</v>
       </c>
       <c r="E295" t="str">
-        <v/>
-      </c>
-      <c r="F295" t="str">
-        <v/>
+        <v>YAK 215N, Air/Hydraulic 2-Stage Trolley Jack (40/20T)</v>
+      </c>
+      <c r="F295" t="str" xml:space="preserve">
+        <v xml:space="preserve">Air / Hydraulic lifting system for all kinds of heavy transport vehicles_x000d_
+Piston is retracted automatically_x000d_
+Dual Descent valve ensures constant and controlled speed under load and increased speed when under load_x000d_
+Heavy duty construction_x000d_
+First Stage: 72 mm second Stage: 78 mm combined: 150 mm _x000d_
+3 piece extension set:_x000d_
+ 1 x 70mm extension_x000d_
+ 1 x 120mm extension_x000d_
+ 1 x 15mm Top Cap</v>
       </c>
       <c r="G295" t="str">
         <v>jacking-lifting</v>
@@ -16099,10 +16107,17 @@
         <v>Y</v>
       </c>
       <c r="P295" t="str">
-        <v>N</v>
-      </c>
-      <c r="Q295" t="str">
-        <v/>
+        <v>Y</v>
+      </c>
+      <c r="Q295" t="str" xml:space="preserve">
+        <v xml:space="preserve">Dimensions: 525 x 300mm_x000d_
+Lifting Capacity: 40/20T_x000d_
+Weight: 39kg_x000d_
+Lift: 72mm + 78mm (150mm)_x000d_
+Manufacturer Part Number: YAK215N_x000d_
+Maximum Lifting Height: 505mm_x000d_
+Minimum Height: 150mm_x000d_
+Operating Pressure: 116-174psi</v>
       </c>
     </row>
     <row r="296">

</xml_diff>